<commit_message>
Update master Excel driver
</commit_message>
<xml_diff>
--- a/Suslife_master_driver.xlsx
+++ b/Suslife_master_driver.xlsx
@@ -342,7 +342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J187"/>
+  <dimension ref="A1:J188"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7372,7 +7372,6 @@
           <t>PERSONAL_NORM</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7388,7 +7387,6 @@
           <t>Koen, että minulla on henkilökohtainen velvollisuus lajitella jätteet huolellisesti.</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
         <v>0</v>
       </c>
@@ -7412,7 +7410,6 @@
           <t>PERSONAL_NORM</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7428,7 +7425,6 @@
           <t>Tuntisin toimivani väärin, jos en lajittelisi jätteitä silloin kun se on mahdollista.</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
       <c r="H177" t="n">
         <v>0</v>
       </c>
@@ -7452,7 +7448,6 @@
           <t>PERSONAL_NORM</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7468,7 +7463,6 @@
           <t>Jätteiden lajittelu on minulle moraalisesti oikea tapa toimia.</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
         <v>0</v>
       </c>
@@ -7492,7 +7486,6 @@
           <t>SELF_IDENTITY</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7508,7 +7501,6 @@
           <t>Pidän itseäni ihmisenä, joka lajittelee jätteet huolellisesti.</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
         <v>0</v>
       </c>
@@ -7532,7 +7524,6 @@
           <t>SELF_IDENTITY</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7548,7 +7539,6 @@
           <t>Jätteiden lajittelu kuuluu siihen, millainen ihminen haluan olla.</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
         <v>0</v>
       </c>
@@ -7572,7 +7562,6 @@
           <t>SELF_IDENTITY</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7588,7 +7577,6 @@
           <t>On minulle tärkeää nähdä itseni ympäristövastuullisena toimijana.</t>
         </is>
       </c>
-      <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
         <v>0</v>
       </c>
@@ -7612,7 +7600,6 @@
           <t>PLAN_CTRL</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7628,7 +7615,6 @@
           <t>Minulla on selkeä suunnitelma siitä, milloin vien lajitellut jätteet eteenpäin.</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
         <v>0</v>
       </c>
@@ -7652,7 +7638,6 @@
           <t>PLAN_CTRL</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7668,7 +7653,6 @@
           <t>Tiedän etukäteen, miten toimin, vaikka arjessa olisi kiire.</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr"/>
       <c r="H183" t="n">
         <v>0</v>
       </c>
@@ -7692,7 +7676,6 @@
           <t>PLAN_CTRL</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7708,7 +7691,6 @@
           <t>Jos lajittelutilanne tulee yllättäen, minulla on valmis toimintatapa.</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
         <v>0</v>
       </c>
@@ -7732,7 +7714,6 @@
           <t>NORM_EXP_G</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7748,7 +7729,6 @@
           <t>Näen usein, että muut ihmiset lajittelevat jätteitä omalla alueellani.</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
         <v>0</v>
       </c>
@@ -7772,7 +7752,6 @@
           <t>NORM_EXP_G</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7788,7 +7767,6 @@
           <t>Taloyhtiössäni tai naapurustossani lajittelu on näkyvä ja tavallinen käytäntö.</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
         <v>0</v>
       </c>
@@ -7812,7 +7790,6 @@
           <t>NORM_EXP_G</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr">
         <is>
           <t>radio</t>
@@ -7828,7 +7805,6 @@
           <t>Lähipiirissäni jätteiden lajittelu on yleistä.</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
         <v>0</v>
       </c>
@@ -7838,6 +7814,49 @@
       <c r="J187" t="inlineStr">
         <is>
           <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>BIO_SORT_PCT</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>bio</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Arvio: kuinka suuri osuus biojätteestä tulee viikon aikana lajiteltua erikseen tai kompostoitua?</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>0–100 %. Vedä liukusäädintä.</t>
+        </is>
+      </c>
+      <c r="H188" t="n">
+        <v>0</v>
+      </c>
+      <c r="I188" t="n">
+        <v>1</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>anchor</t>
         </is>
       </c>
     </row>
@@ -12222,7 +12241,6 @@
           <t>PERSONAL_NORM</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>Henkilökohtainen velvollisuus</t>
@@ -12256,7 +12274,6 @@
           <t>PERSONAL_NORM</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>Henkilökohtainen velvollisuus</t>
@@ -12290,7 +12307,6 @@
           <t>PERSONAL_NORM</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>Henkilökohtainen velvollisuus</t>
@@ -12324,7 +12340,6 @@
           <t>SELF_IDENTITY</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>Lajittelijaidentiteetti</t>
@@ -12358,7 +12373,6 @@
           <t>SELF_IDENTITY</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>Lajittelijaidentiteetti</t>
@@ -12392,7 +12406,6 @@
           <t>SELF_IDENTITY</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>Lajittelijaidentiteetti</t>
@@ -12426,7 +12439,6 @@
           <t>PLAN_CTRL</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>Suunnittelu / action control</t>
@@ -12460,7 +12472,6 @@
           <t>PLAN_CTRL</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>Suunnittelu / action control</t>
@@ -12494,7 +12505,6 @@
           <t>PLAN_CTRL</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>Suunnittelu / action control</t>
@@ -12528,7 +12538,6 @@
           <t>NORM_EXP_G</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>Lajittelun näkyvyys lähiympäristössä</t>
@@ -12562,7 +12571,6 @@
           <t>NORM_EXP_G</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>Lajittelun näkyvyys lähiympäristössä</t>
@@ -12596,7 +12604,6 @@
           <t>NORM_EXP_G</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>Lajittelun näkyvyys lähiympäristössä</t>
@@ -12856,7 +12863,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SORT_F|PL_UNSORT_PCT|SQ2|SQ3|INT1|INT3|HAB2|HAB3|CAP1|CAP2|SOC1|SOC2|SOC3|TRUST1|TRUST2|TRUST3</t>
+          <t>SORT_F|PL_UNSORT_PCT|PL_ANCHOR_OE|SQ2|SQ3|INT1|INT3|HAB2|HAB3|CAP1|CAP2|SOC1|SOC2|SOC3|TRUST1|TRUST2|TRUST3</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -13067,7 +13074,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BIO_SORT_F|BIO_SQ2|BIO_SQ3|BIO_INT1|BIO_INT3|BIO_HAB2|BIO_HAB3|BIO_CAP1|BIO_CAP2|BIO_PBC1|BIO_PBC2|BIO_CLAR1|BIO_CLAR3|BIO_YF1|BIO_YF3</t>
+          <t>BIO_SORT_F|BIO_SORT_PCT|BIO_ANCHOR_OE|BIO_SQ2|BIO_SQ3|BIO_INT1|BIO_INT3|BIO_HAB2|BIO_HAB3|BIO_CAP1|BIO_CAP2|BIO_PBC1|BIO_PBC2|BIO_CLAR1|BIO_CLAR3|BIO_YF1|BIO_YF3</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -13271,7 +13278,6 @@
           <t>Henkilökohtainen velvollisuus ja identiteetti</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>PERSONAL_NORM1|PERSONAL_NORM2|PERSONAL_NORM3|SELF_IDENTITY1|SELF_IDENTITY2|SELF_IDENTITY3</t>
@@ -13300,7 +13306,6 @@
           <t>Suunnittelu ja lajittelun näkyvyys</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>PLAN_CTRL1|PLAN_CTRL2|PLAN_CTRL3|NORM_EXP_G1|NORM_EXP_G2|NORM_EXP_G3</t>
@@ -13329,7 +13334,6 @@
           <t>Mieltymykset selkeyteen</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>INSTR_NFC_G|NFC_G1|NFC_G2|NFC_G3|NFC_G4|NFC_G5|NFC_G6</t>
@@ -13358,7 +13362,6 @@
           <t>Arvot</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>INSTR_VALUES|VAL_BIOS1|VAL_BIOS2|VAL_BIOS3|VAL_BIOS4|VAL_ALTR1|VAL_ALTR2|VAL_ALTR3|VAL_ALTR4|VAL_EGO1|VAL_EGO2|VAL_EGO3|VAL_HED1|VAL_HED2</t>
@@ -13387,7 +13390,6 @@
           <t>Yleinen suhtautuminen ohjaamiseen</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>REACT</t>
@@ -18585,9 +18587,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update master sheet and intro image
</commit_message>
<xml_diff>
--- a/Suslife_master_driver.xlsx
+++ b/Suslife_master_driver.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twttom/Documents/sustlife_survey_demo/BUILD2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5CE873-C082-D240-9C9A-C220A2B30847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2050D9D8-11B3-AA4C-B43F-80F32E3F9817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="760" windowWidth="34560" windowHeight="20660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="760" windowWidth="34560" windowHeight="20660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ITEMS" sheetId="1" r:id="rId1"/>
@@ -3481,17 +3481,17 @@
     <t>v5 update: plastic/bio core flow rebuilt to latest main-spec item lists; info-type ranking block added; repeated HOUSING and Q_COMPOST removed from main-survey infrastructure page.</t>
   </si>
   <si>
-    <t>"/media/introb.png
-## Biojäte
-Biojäte on maatuvaa ja kompostoituvaa jätettä, johon kuuluu erityisesti ruoka- ja keittiöjätettä, kuten hedelmien ja vihannesten kuoria, ruoantähteitä, kahvinporoja ja teepusseja. EU:n jätedirektiivin mukaan biojätteeseen luetaan myös biohajoava puutarha- ja puistojäte sekä kotitalouksista, ravintoloista, toimistoista ja muista vastaavista toiminnoista syntyvä elintarvike- ja keittiöjäte. Kotitalouksissa biojätteen lajittelu vähentää sekajätteen määrää ja mahdollistaa jätteen hyödyntämisen esimerkiksi kompostina ja biokaasun tuotannossa. Suomessa biojätteen erilliskeräystä on laajennettu vaiheittain, ja sen voi tietyin ehdoin korvata kiinteistöllä tapahtuvalla kompostoinnilla. Biojätteen kierrätys edistää ravinteiden kiertoa, vähentää jätteen polttoon ja sekajätteeseen päätyvän orgaanisen aineksen määrää sekä tukee kiertotaloutta."</t>
-  </si>
-  <si>
     <t>![](/media/vignettes_labeled/971790_028.png)
 Kuvittele, että tämä ratkaisu otetaan käyttöön omalla alueellasi.
 Keräyspisteessä kerrotaan selkeästi,
 miten biojäte hyödynnetään paikallisesti esimerkiksi biokaasuna ja lannoitteena.
 Läpinäkyvä tieto vahvistaa luottamusta siihen,
 että biojätteen lajittelu on hyödyllistä.</t>
+  </si>
+  <si>
+    <t>/media/introb.png
+## Biojäte
+Biojäte on maatuvaa ja kompostoituvaa jätettä, johon kuuluu erityisesti ruoka- ja keittiöjätettä, kuten hedelmien ja vihannesten kuoria, ruoantähteitä, kahvinporoja ja teepusseja. EU:n jätedirektiivin mukaan biojätteeseen luetaan myös biohajoava puutarha- ja puistojäte sekä kotitalouksista, ravintoloista, toimistoista ja muista vastaavista toiminnoista syntyvä elintarvike- ja keittiöjäte. Kotitalouksissa biojätteen lajittelu vähentää sekajätteen määrää ja mahdollistaa jätteen hyödyntämisen esimerkiksi kompostina ja biokaasun tuotannossa. Suomessa biojätteen erilliskeräystä on laajennettu vaiheittain, ja sen voi tietyin ehdoin korvata kiinteistöllä tapahtuvalla kompostoinnilla. Biojätteen kierrätys edistää ravinteiden kiertoa, vähentää jätteen polttoon ja sekajätteeseen päätyvän orgaanisen aineksen määrää sekä tukee kiertotaloutta.</t>
   </si>
 </sst>
 </file>
@@ -4428,7 +4428,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>82</v>
       </c>
@@ -4438,7 +4438,7 @@
       <c r="D26" t="s">
         <v>83</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="3" t="s">
         <v>84</v>
       </c>
       <c r="H26">
@@ -4462,7 +4462,7 @@
         <v>83</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="H27">
         <v>0</v>
@@ -15653,7 +15653,7 @@
         <v>938</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="G47">
         <v>1</v>

</xml_diff>

<commit_message>
Update app and master driver
</commit_message>
<xml_diff>
--- a/Suslife_master_driver.xlsx
+++ b/Suslife_master_driver.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twttom/Documents/sustlife_survey_demo/BUILD2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40AA9FC5-2193-FA4B-A40A-1B73045D36D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C542FD-CE4A-B646-A479-594A49071E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="760" windowWidth="34560" windowHeight="20620" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="760" windowWidth="34560" windowHeight="20620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ITEMS" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="1102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3048" uniqueCount="1103">
   <si>
     <t>item_id</t>
   </si>
@@ -3624,6 +3624,16 @@
   </si>
   <si>
     <t>v5 update: plastic/bio core flow rebuilt to latest main-spec item lists; info-type ranking block added; repeated HOUSING and Q_COMPOST removed from main-survey infrastructure page.</t>
+  </si>
+  <si>
+    <t>![](/media/vignettes_labeled/971790_035.png)
+Kuvittele, että tämä ratkaisu otetaan käyttöön omalla alueellasi.
+Jätehuoneessa on ilmoitustaulu, jossa kerrotaan taloyhtiön muovipakkausten lajittelun tuloksista. Taulussa näkyy esimerkiksi:
+• kuinka paljon muovia on kerätty viime kuussa  
+• miten lajittelun laatu on kehittynyt  
+• vertailu edelliseen kuukauteen tai lähialueen keskiarvoon  
+Taulussa kerrotaan myös lyhyesti, mihin lajiteltu muovi päätyy (esim. uusiomuoviksi uusien tuotteiden valmistukseen).
+Ratkaisu tekee lajittelun tulokset näkyviksi ja voi kannustaa lajittelemaan muovia entistä huolellisemmin.</t>
   </si>
 </sst>
 </file>
@@ -14504,7 +14514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="224" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>881</v>
       </c>
@@ -14544,7 +14554,7 @@
       <c r="T6" t="s">
         <v>886</v>
       </c>
-      <c r="U6" t="s">
+      <c r="U6" s="3" t="s">
         <v>883</v>
       </c>
       <c r="V6">
@@ -14588,6 +14598,15 @@
       <c r="N7">
         <v>0</v>
       </c>
+      <c r="T7" s="3" t="s">
+        <v>1102</v>
+      </c>
+      <c r="U7" s="3" t="s">
+        <v>1102</v>
+      </c>
+      <c r="V7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -15042,6 +15061,15 @@
       </c>
       <c r="N17">
         <v>0</v>
+      </c>
+      <c r="T17" s="3" t="s">
+        <v>1102</v>
+      </c>
+      <c r="U17" s="3" t="s">
+        <v>1102</v>
+      </c>
+      <c r="V17">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update app, sheet, and labeled images
</commit_message>
<xml_diff>
--- a/Suslife_master_driver.xlsx
+++ b/Suslife_master_driver.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twttom/Documents/sustlife_survey_demo/BUILD2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB9BE021-989F-7F4C-862B-EABDFFA3E2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82166186-3EAB-B945-9B17-C7ED1A530891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="760" windowWidth="16640" windowHeight="20660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="760" windowWidth="16640" windowHeight="20660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ITEMS" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3082" uniqueCount="1129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3100" uniqueCount="1143">
   <si>
     <t>item_id</t>
   </si>
@@ -3733,6 +3733,52 @@
     <t>![](/media/vignettes_labeled/971790_043.png) Kuvittele, että tämä ratkaisu otetaan käyttöön omalla alueellasi.
 Taloyhtiö tai alue tarjoaa asukkaille mahdollisuuden tilata bioastian tai kompostorin helposti yhteishankintana.
 Yhteinen tilaus madaltaa aloittamisen kynnystä ja tekee biojätteen lajittelun aloittamisesta helpompaa.</t>
+  </si>
+  <si>
+    <t>DET_RU_BIO_B19</t>
+  </si>
+  <si>
+    <t>Kyläkohtainen palaute sekajätteen sisällöstä</t>
+  </si>
+  <si>
+    <t>BioA19</t>
+  </si>
+  <si>
+    <t>area_feedback / contamination_salience</t>
+  </si>
+  <si>
+    <t>Resident in a rural Finnish detached-house yard reading a waste-company letter about mixed-waste composition, simple chart visible, household bins nearby, documentary style.</t>
+  </si>
+  <si>
+    <t>NEW_DET_RU_BIO_B19.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ![](/media/vignettes_labeled/971790_044.png) Kuvittele, että tämä ratkaisu otetaan käyttöön omalla alueellasi.
+Saat kirjeen tai tiedotteen, jossa kerrotaan oman alueen sekajätteen koostumustutkimuksen tuloksista. Viestissä näytetään, kuinka paljon biojätettä on edelleen sekajätteen joukossa ja miksi sen vähentäminen on tärkeää.
+Palaute tekee lajittelun vaikutukset näkyviksi ja auttaa vähentämään biojätteen päätymistä sekajätteeseen.</t>
+  </si>
+  <si>
+    <t>DET_RU_PL_A24</t>
+  </si>
+  <si>
+    <t>Muovinkeräyksen kokeilupaketti kotiin</t>
+  </si>
+  <si>
+    <t>A24</t>
+  </si>
+  <si>
+    <t>Rural Finnish detached-house yard with a simple plastic sorting starter kit and leaflet, practical countryside environment, documentary style.</t>
+  </si>
+  <si>
+    <t>NEW_DET_RU_PL_A24.png</t>
+  </si>
+  <si>
+    <t>enablement ,starter_pack / habit_support</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ![](/media/vignettes_labeled/971790_045.png) Kuvittele, että tämä ratkaisu otetaan käyttöön omalla alueellasi.
+Kotitalous saa kokeilupaketin muovipakkausten lajittelun aloittamiseen. Paketti sisältää keräysastian, lyhyet ohjeet ja tiedon siitä, miten lajittelua voi kokeilla helposti arjessa.
+Kokeilupaketti madaltaa aloittamisen kynnystä ja auttaa rakentamaan uutta lajittelurutiinia.</t>
   </si>
 </sst>
 </file>
@@ -14366,7 +14412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:V66"/>
+  <dimension ref="A1:V68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
@@ -15808,106 +15854,91 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>978</v>
+        <v>1136</v>
       </c>
       <c r="B32" t="s">
-        <v>979</v>
+        <v>934</v>
       </c>
       <c r="C32" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D32" t="s">
-        <v>949</v>
-      </c>
-      <c r="E32" t="s">
-        <v>950</v>
+        <v>1137</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>1142</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>951</v>
+        <v>1138</v>
       </c>
       <c r="I32" t="s">
-        <v>980</v>
+        <v>1141</v>
+      </c>
+      <c r="J32" t="s">
+        <v>1139</v>
       </c>
       <c r="K32" t="s">
-        <v>858</v>
-      </c>
-      <c r="L32" t="s">
-        <v>775</v>
-      </c>
-      <c r="M32" t="s">
-        <v>986</v>
-      </c>
-      <c r="N32">
-        <v>0</v>
-      </c>
-      <c r="T32" s="3" t="s">
-        <v>987</v>
-      </c>
-      <c r="U32" s="3" t="s">
-        <v>983</v>
-      </c>
-      <c r="V32" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>981</v>
+        <v>1129</v>
       </c>
       <c r="B33" t="s">
-        <v>979</v>
+        <v>934</v>
       </c>
       <c r="C33" t="s">
         <v>24</v>
       </c>
       <c r="D33" t="s">
-        <v>982</v>
+        <v>1130</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>1135</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1131</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33" t="s">
+        <v>1132</v>
+      </c>
+      <c r="I33" t="s">
+        <v>1133</v>
+      </c>
+      <c r="J33" t="s">
+        <v>1134</v>
+      </c>
+      <c r="K33" t="s">
+        <v>775</v>
+      </c>
+      <c r="L33" t="s">
+        <v>986</v>
+      </c>
+      <c r="M33">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3" t="s">
+        <v>987</v>
+      </c>
+      <c r="U33" s="3" t="s">
         <v>983</v>
       </c>
-      <c r="G33">
-        <v>1</v>
-      </c>
-      <c r="H33" t="s">
-        <v>984</v>
-      </c>
-      <c r="I33" t="s">
-        <v>985</v>
-      </c>
-      <c r="K33" t="s">
-        <v>858</v>
-      </c>
-      <c r="L33" t="s">
-        <v>775</v>
-      </c>
-      <c r="M33" t="s">
-        <v>991</v>
-      </c>
-      <c r="N33">
-        <v>0</v>
-      </c>
-      <c r="O33">
-        <v>1</v>
-      </c>
-      <c r="T33" t="s">
-        <v>992</v>
-      </c>
-      <c r="U33" t="s">
-        <v>989</v>
-      </c>
-      <c r="V33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>988</v>
+        <v>978</v>
       </c>
       <c r="B34" t="s">
         <v>979</v>
@@ -15916,19 +15947,19 @@
         <v>24</v>
       </c>
       <c r="D34" t="s">
-        <v>862</v>
+        <v>949</v>
       </c>
       <c r="E34" t="s">
-        <v>989</v>
+        <v>950</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>864</v>
+        <v>951</v>
       </c>
       <c r="I34" t="s">
-        <v>990</v>
+        <v>980</v>
       </c>
       <c r="K34" t="s">
         <v>858</v>
@@ -15937,45 +15968,48 @@
         <v>775</v>
       </c>
       <c r="M34" t="s">
-        <v>905</v>
+        <v>991</v>
       </c>
       <c r="N34">
         <v>0</v>
       </c>
-      <c r="T34" s="3" t="s">
-        <v>996</v>
-      </c>
-      <c r="U34" s="3" t="s">
-        <v>994</v>
-      </c>
-      <c r="V34" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="O34">
+        <v>1</v>
+      </c>
+      <c r="T34" t="s">
+        <v>992</v>
+      </c>
+      <c r="U34" t="s">
+        <v>989</v>
+      </c>
+      <c r="V34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>993</v>
+        <v>981</v>
       </c>
       <c r="B35" t="s">
         <v>979</v>
       </c>
       <c r="C35" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D35" t="s">
-        <v>974</v>
+        <v>982</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>994</v>
+        <v>983</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>976</v>
+        <v>984</v>
       </c>
       <c r="I35" t="s">
-        <v>995</v>
+        <v>985</v>
       </c>
       <c r="K35" t="s">
         <v>858</v>
@@ -15984,42 +16018,45 @@
         <v>775</v>
       </c>
       <c r="M35" t="s">
-        <v>1001</v>
+        <v>905</v>
       </c>
       <c r="N35">
         <v>0</v>
       </c>
-      <c r="O35" t="s">
-        <v>1002</v>
-      </c>
-      <c r="Q35" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T35" s="3" t="s">
+        <v>996</v>
+      </c>
+      <c r="U35" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="V35" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="B36" t="s">
         <v>979</v>
       </c>
       <c r="C36" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D36" t="s">
-        <v>998</v>
+        <v>862</v>
       </c>
       <c r="E36" t="s">
-        <v>999</v>
+        <v>989</v>
       </c>
       <c r="G36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>890</v>
+        <v>864</v>
       </c>
       <c r="I36" t="s">
-        <v>1000</v>
+        <v>990</v>
       </c>
       <c r="K36" t="s">
         <v>858</v>
@@ -16028,27 +16065,21 @@
         <v>775</v>
       </c>
       <c r="M36" t="s">
-        <v>1009</v>
+        <v>1001</v>
       </c>
       <c r="N36">
         <v>0</v>
       </c>
-      <c r="O36">
-        <v>1</v>
-      </c>
-      <c r="T36" s="3" t="s">
-        <v>1010</v>
-      </c>
-      <c r="U36" s="3" t="s">
-        <v>1006</v>
-      </c>
-      <c r="V36" s="3">
-        <v>1</v>
+      <c r="O36" t="s">
+        <v>1002</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>1003</v>
       </c>
     </row>
     <row r="37" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>1004</v>
+        <v>993</v>
       </c>
       <c r="B37" t="s">
         <v>979</v>
@@ -16057,19 +16088,19 @@
         <v>30</v>
       </c>
       <c r="D37" t="s">
-        <v>1005</v>
+        <v>974</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>1006</v>
+        <v>994</v>
       </c>
       <c r="G37">
         <v>1</v>
       </c>
       <c r="H37" t="s">
-        <v>1007</v>
+        <v>976</v>
       </c>
       <c r="I37" t="s">
-        <v>1008</v>
+        <v>995</v>
       </c>
       <c r="K37" t="s">
         <v>858</v>
@@ -16077,16 +16108,28 @@
       <c r="L37" t="s">
         <v>775</v>
       </c>
-      <c r="O37" t="s">
-        <v>1015</v>
-      </c>
-      <c r="S37">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="M37" t="s">
+        <v>1009</v>
+      </c>
+      <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <v>1</v>
+      </c>
+      <c r="T37" s="3" t="s">
+        <v>1010</v>
+      </c>
+      <c r="U37" s="3" t="s">
+        <v>1006</v>
+      </c>
+      <c r="V37" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>1011</v>
+        <v>997</v>
       </c>
       <c r="B38" t="s">
         <v>979</v>
@@ -16095,19 +16138,19 @@
         <v>30</v>
       </c>
       <c r="D38" t="s">
-        <v>1012</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>1013</v>
+        <v>998</v>
+      </c>
+      <c r="E38" t="s">
+        <v>999</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" t="s">
-        <v>1014</v>
+        <v>890</v>
       </c>
       <c r="I38" t="s">
-        <v>990</v>
+        <v>1000</v>
       </c>
       <c r="K38" t="s">
         <v>858</v>
@@ -16115,25 +16158,16 @@
       <c r="L38" t="s">
         <v>775</v>
       </c>
-      <c r="M38" t="s">
-        <v>1020</v>
-      </c>
-      <c r="N38">
-        <v>0</v>
-      </c>
-      <c r="T38" t="s">
-        <v>1021</v>
-      </c>
-      <c r="U38" t="s">
-        <v>1018</v>
-      </c>
-      <c r="V38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="O38" t="s">
+        <v>1015</v>
+      </c>
+      <c r="S38">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>1016</v>
+        <v>1004</v>
       </c>
       <c r="B39" t="s">
         <v>979</v>
@@ -16142,19 +16176,19 @@
         <v>30</v>
       </c>
       <c r="D39" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E39" t="s">
-        <v>1018</v>
+        <v>1005</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>1006</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>1019</v>
+        <v>1007</v>
       </c>
       <c r="I39" t="s">
-        <v>878</v>
+        <v>1008</v>
       </c>
       <c r="K39" t="s">
         <v>858</v>
@@ -16163,45 +16197,45 @@
         <v>775</v>
       </c>
       <c r="M39" t="s">
-        <v>946</v>
+        <v>1020</v>
       </c>
       <c r="N39">
         <v>0</v>
       </c>
       <c r="T39" t="s">
-        <v>947</v>
+        <v>1021</v>
       </c>
       <c r="U39" t="s">
-        <v>943</v>
+        <v>1018</v>
       </c>
       <c r="V39">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>1022</v>
+        <v>1011</v>
       </c>
       <c r="B40" t="s">
-        <v>1023</v>
+        <v>979</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D40" t="s">
-        <v>942</v>
-      </c>
-      <c r="E40" t="s">
-        <v>943</v>
+        <v>1012</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>1013</v>
       </c>
       <c r="G40">
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>944</v>
+        <v>1014</v>
       </c>
       <c r="I40" t="s">
-        <v>945</v>
+        <v>990</v>
       </c>
       <c r="K40" t="s">
         <v>858</v>
@@ -16210,45 +16244,45 @@
         <v>775</v>
       </c>
       <c r="M40" t="s">
-        <v>991</v>
+        <v>946</v>
       </c>
       <c r="N40">
         <v>0</v>
       </c>
       <c r="T40" t="s">
-        <v>992</v>
+        <v>947</v>
       </c>
       <c r="U40" t="s">
-        <v>989</v>
+        <v>943</v>
       </c>
       <c r="V40">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>1024</v>
+        <v>1016</v>
       </c>
       <c r="B41" t="s">
-        <v>1023</v>
+        <v>979</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D41" t="s">
-        <v>862</v>
+        <v>1017</v>
       </c>
       <c r="E41" t="s">
-        <v>989</v>
+        <v>1018</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41" t="s">
-        <v>864</v>
+        <v>1019</v>
       </c>
       <c r="I41" t="s">
-        <v>865</v>
+        <v>878</v>
       </c>
       <c r="K41" t="s">
         <v>858</v>
@@ -16257,21 +16291,24 @@
         <v>775</v>
       </c>
       <c r="M41" t="s">
-        <v>859</v>
+        <v>991</v>
       </c>
       <c r="N41">
         <v>0</v>
       </c>
-      <c r="O41">
-        <v>1</v>
-      </c>
-      <c r="P41" t="s">
-        <v>1028</v>
-      </c>
-    </row>
-    <row r="42" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="T41" t="s">
+        <v>992</v>
+      </c>
+      <c r="U41" t="s">
+        <v>989</v>
+      </c>
+      <c r="V41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>1025</v>
+        <v>1022</v>
       </c>
       <c r="B42" t="s">
         <v>1023</v>
@@ -16280,19 +16317,19 @@
         <v>24</v>
       </c>
       <c r="D42" t="s">
-        <v>854</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>1026</v>
+        <v>942</v>
+      </c>
+      <c r="E42" t="s">
+        <v>943</v>
       </c>
       <c r="G42">
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>856</v>
+        <v>944</v>
       </c>
       <c r="I42" t="s">
-        <v>1027</v>
+        <v>945</v>
       </c>
       <c r="K42" t="s">
         <v>858</v>
@@ -16301,24 +16338,21 @@
         <v>775</v>
       </c>
       <c r="M42" t="s">
-        <v>885</v>
+        <v>859</v>
       </c>
       <c r="N42">
         <v>0</v>
       </c>
-      <c r="T42" t="s">
-        <v>886</v>
-      </c>
-      <c r="U42" t="s">
-        <v>958</v>
-      </c>
-      <c r="V42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="O42">
+        <v>1</v>
+      </c>
+      <c r="P42" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>1029</v>
+        <v>1024</v>
       </c>
       <c r="B43" t="s">
         <v>1023</v>
@@ -16327,19 +16361,19 @@
         <v>24</v>
       </c>
       <c r="D43" t="s">
-        <v>882</v>
+        <v>862</v>
       </c>
       <c r="E43" t="s">
-        <v>958</v>
+        <v>989</v>
       </c>
       <c r="G43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H43" t="s">
-        <v>884</v>
+        <v>864</v>
       </c>
       <c r="I43" t="s">
-        <v>878</v>
+        <v>865</v>
       </c>
       <c r="K43" t="s">
         <v>858</v>
@@ -16348,45 +16382,45 @@
         <v>775</v>
       </c>
       <c r="M43" t="s">
-        <v>905</v>
+        <v>885</v>
       </c>
       <c r="N43">
         <v>0</v>
       </c>
-      <c r="T43" s="3" t="s">
-        <v>1031</v>
-      </c>
-      <c r="U43" s="3" t="s">
-        <v>994</v>
-      </c>
-      <c r="V43" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="T43" t="s">
+        <v>886</v>
+      </c>
+      <c r="U43" t="s">
+        <v>958</v>
+      </c>
+      <c r="V43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>1030</v>
+        <v>1025</v>
       </c>
       <c r="B44" t="s">
         <v>1023</v>
       </c>
       <c r="C44" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D44" t="s">
-        <v>974</v>
+        <v>854</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>994</v>
+        <v>1026</v>
       </c>
       <c r="G44">
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>976</v>
+        <v>856</v>
       </c>
       <c r="I44" t="s">
-        <v>995</v>
+        <v>1027</v>
       </c>
       <c r="K44" t="s">
         <v>858</v>
@@ -16395,36 +16429,45 @@
         <v>775</v>
       </c>
       <c r="M44" t="s">
-        <v>1001</v>
+        <v>905</v>
       </c>
       <c r="N44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T44" s="3" t="s">
+        <v>1031</v>
+      </c>
+      <c r="U44" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="V44" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
       <c r="B45" t="s">
         <v>1023</v>
       </c>
       <c r="C45" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D45" t="s">
-        <v>998</v>
+        <v>882</v>
       </c>
       <c r="E45" t="s">
-        <v>999</v>
+        <v>958</v>
       </c>
       <c r="G45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H45" t="s">
-        <v>890</v>
+        <v>884</v>
       </c>
       <c r="I45" t="s">
-        <v>1000</v>
+        <v>878</v>
       </c>
       <c r="K45" t="s">
         <v>858</v>
@@ -16433,27 +16476,15 @@
         <v>775</v>
       </c>
       <c r="M45" t="s">
-        <v>1020</v>
+        <v>1001</v>
       </c>
       <c r="N45">
         <v>0</v>
       </c>
-      <c r="O45">
-        <v>1</v>
-      </c>
-      <c r="T45" s="3" t="s">
-        <v>1035</v>
-      </c>
-      <c r="U45" s="3" t="s">
-        <v>1034</v>
-      </c>
-      <c r="V45" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="B46" t="s">
         <v>1023</v>
@@ -16462,19 +16493,19 @@
         <v>30</v>
       </c>
       <c r="D46" t="s">
-        <v>894</v>
+        <v>974</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>1034</v>
+        <v>994</v>
       </c>
       <c r="G46">
         <v>1</v>
       </c>
       <c r="H46" t="s">
-        <v>896</v>
+        <v>976</v>
       </c>
       <c r="I46" t="s">
-        <v>897</v>
+        <v>995</v>
       </c>
       <c r="K46" t="s">
         <v>858</v>
@@ -16488,19 +16519,22 @@
       <c r="N46">
         <v>0</v>
       </c>
-      <c r="T46" t="s">
-        <v>1021</v>
-      </c>
-      <c r="U46" t="s">
-        <v>1018</v>
-      </c>
-      <c r="V46">
+      <c r="O46">
+        <v>1</v>
+      </c>
+      <c r="T46" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="U46" s="3" t="s">
+        <v>1034</v>
+      </c>
+      <c r="V46" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="B47" t="s">
         <v>1023</v>
@@ -16509,19 +16543,19 @@
         <v>30</v>
       </c>
       <c r="D47" t="s">
-        <v>1017</v>
+        <v>998</v>
       </c>
       <c r="E47" t="s">
-        <v>1018</v>
+        <v>999</v>
       </c>
       <c r="G47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>1019</v>
+        <v>890</v>
       </c>
       <c r="I47" t="s">
-        <v>878</v>
+        <v>1000</v>
       </c>
       <c r="K47" t="s">
         <v>858</v>
@@ -16530,24 +16564,24 @@
         <v>775</v>
       </c>
       <c r="M47" t="s">
-        <v>1042</v>
+        <v>1020</v>
       </c>
       <c r="N47">
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>1043</v>
+        <v>1021</v>
       </c>
       <c r="U47" t="s">
-        <v>1039</v>
+        <v>1018</v>
       </c>
       <c r="V47">
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="B48" t="s">
         <v>1023</v>
@@ -16556,19 +16590,19 @@
         <v>30</v>
       </c>
       <c r="D48" t="s">
-        <v>1038</v>
-      </c>
-      <c r="E48" t="s">
-        <v>1039</v>
+        <v>894</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>1034</v>
       </c>
       <c r="G48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>1040</v>
+        <v>896</v>
       </c>
       <c r="I48" t="s">
-        <v>1041</v>
+        <v>897</v>
       </c>
       <c r="K48" t="s">
         <v>858</v>
@@ -16577,45 +16611,45 @@
         <v>775</v>
       </c>
       <c r="M48" t="s">
-        <v>986</v>
+        <v>1042</v>
       </c>
       <c r="N48">
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="U48" t="s">
-        <v>1048</v>
+        <v>1039</v>
       </c>
       <c r="V48">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="B49" t="s">
-        <v>1045</v>
+        <v>1023</v>
       </c>
       <c r="C49" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D49" t="s">
-        <v>982</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>1046</v>
+        <v>1017</v>
+      </c>
+      <c r="E49" t="s">
+        <v>1018</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H49" t="s">
-        <v>984</v>
+        <v>1019</v>
       </c>
       <c r="I49" t="s">
-        <v>985</v>
+        <v>878</v>
       </c>
       <c r="K49" t="s">
         <v>858</v>
@@ -16624,16 +16658,16 @@
         <v>775</v>
       </c>
       <c r="M49" t="s">
-        <v>991</v>
+        <v>986</v>
       </c>
       <c r="N49">
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>992</v>
+        <v>1047</v>
       </c>
       <c r="U49" t="s">
-        <v>989</v>
+        <v>1048</v>
       </c>
       <c r="V49">
         <v>1</v>
@@ -16641,28 +16675,28 @@
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>1049</v>
+        <v>1037</v>
       </c>
       <c r="B50" t="s">
-        <v>1045</v>
+        <v>1023</v>
       </c>
       <c r="C50" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D50" t="s">
-        <v>862</v>
+        <v>1038</v>
       </c>
       <c r="E50" t="s">
-        <v>989</v>
+        <v>1039</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50" t="s">
-        <v>864</v>
+        <v>1040</v>
       </c>
       <c r="I50" t="s">
-        <v>865</v>
+        <v>1041</v>
       </c>
       <c r="K50" t="s">
         <v>858</v>
@@ -16671,27 +16705,24 @@
         <v>775</v>
       </c>
       <c r="M50" t="s">
-        <v>953</v>
+        <v>991</v>
       </c>
       <c r="N50">
         <v>0</v>
       </c>
-      <c r="O50">
-        <v>1</v>
-      </c>
       <c r="T50" t="s">
-        <v>954</v>
+        <v>992</v>
       </c>
       <c r="U50" t="s">
-        <v>950</v>
+        <v>989</v>
       </c>
       <c r="V50">
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>1050</v>
+        <v>1044</v>
       </c>
       <c r="B51" t="s">
         <v>1045</v>
@@ -16700,19 +16731,19 @@
         <v>24</v>
       </c>
       <c r="D51" t="s">
-        <v>949</v>
-      </c>
-      <c r="E51" t="s">
-        <v>950</v>
+        <v>982</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>1046</v>
       </c>
       <c r="G51">
         <v>1</v>
       </c>
       <c r="H51" t="s">
-        <v>951</v>
+        <v>984</v>
       </c>
       <c r="I51" t="s">
-        <v>990</v>
+        <v>985</v>
       </c>
       <c r="K51" t="s">
         <v>858</v>
@@ -16721,48 +16752,48 @@
         <v>775</v>
       </c>
       <c r="M51" t="s">
-        <v>1009</v>
+        <v>953</v>
       </c>
       <c r="N51">
         <v>0</v>
       </c>
-      <c r="O51" t="s">
-        <v>1054</v>
+      <c r="O51">
+        <v>1</v>
       </c>
       <c r="T51" t="s">
-        <v>1055</v>
+        <v>954</v>
       </c>
       <c r="U51" t="s">
-        <v>1052</v>
+        <v>950</v>
       </c>
       <c r="V51">
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B52" t="s">
         <v>1045</v>
       </c>
       <c r="C52" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D52" t="s">
-        <v>1005</v>
+        <v>862</v>
       </c>
       <c r="E52" t="s">
-        <v>1052</v>
+        <v>989</v>
       </c>
       <c r="G52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>1007</v>
+        <v>864</v>
       </c>
       <c r="I52" t="s">
-        <v>1053</v>
+        <v>865</v>
       </c>
       <c r="K52" t="s">
         <v>858</v>
@@ -16771,45 +16802,48 @@
         <v>775</v>
       </c>
       <c r="M52" t="s">
-        <v>1058</v>
+        <v>1009</v>
       </c>
       <c r="N52">
         <v>0</v>
       </c>
-      <c r="T52" s="3" t="s">
-        <v>1059</v>
-      </c>
-      <c r="U52" s="3" t="s">
-        <v>1057</v>
-      </c>
-      <c r="V52" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="O52" t="s">
+        <v>1054</v>
+      </c>
+      <c r="T52" t="s">
+        <v>1055</v>
+      </c>
+      <c r="U52" t="s">
+        <v>1052</v>
+      </c>
+      <c r="V52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>1056</v>
+        <v>1050</v>
       </c>
       <c r="B53" t="s">
         <v>1045</v>
       </c>
       <c r="C53" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D53" t="s">
-        <v>974</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>1057</v>
+        <v>949</v>
+      </c>
+      <c r="E53" t="s">
+        <v>950</v>
       </c>
       <c r="G53">
         <v>1</v>
       </c>
       <c r="H53" t="s">
-        <v>976</v>
+        <v>951</v>
       </c>
       <c r="I53" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="K53" t="s">
         <v>858</v>
@@ -16818,19 +16852,16 @@
         <v>775</v>
       </c>
       <c r="M53" t="s">
-        <v>1020</v>
+        <v>1058</v>
       </c>
       <c r="N53">
         <v>0</v>
       </c>
-      <c r="O53">
-        <v>1</v>
-      </c>
       <c r="T53" s="3" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="U53" s="3" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="V53" s="3">
         <v>1</v>
@@ -16838,7 +16869,7 @@
     </row>
     <row r="54" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>1060</v>
+        <v>1051</v>
       </c>
       <c r="B54" t="s">
         <v>1045</v>
@@ -16847,19 +16878,19 @@
         <v>30</v>
       </c>
       <c r="D54" t="s">
-        <v>894</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>1061</v>
+        <v>1005</v>
+      </c>
+      <c r="E54" t="s">
+        <v>1052</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H54" t="s">
-        <v>896</v>
+        <v>1007</v>
       </c>
       <c r="I54" t="s">
-        <v>897</v>
+        <v>1053</v>
       </c>
       <c r="K54" t="s">
         <v>858</v>
@@ -16867,13 +16898,28 @@
       <c r="L54" t="s">
         <v>775</v>
       </c>
-      <c r="O54" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="55" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="M54" t="s">
+        <v>1020</v>
+      </c>
+      <c r="N54">
+        <v>0</v>
+      </c>
+      <c r="O54">
+        <v>1</v>
+      </c>
+      <c r="T54" s="3" t="s">
+        <v>1062</v>
+      </c>
+      <c r="U54" s="3" t="s">
+        <v>1061</v>
+      </c>
+      <c r="V54" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>1063</v>
+        <v>1056</v>
       </c>
       <c r="B55" t="s">
         <v>1045</v>
@@ -16882,19 +16928,19 @@
         <v>30</v>
       </c>
       <c r="D55" t="s">
-        <v>1064</v>
+        <v>974</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="G55">
         <v>1</v>
       </c>
       <c r="H55" t="s">
-        <v>1066</v>
+        <v>976</v>
       </c>
       <c r="I55" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="K55" t="s">
         <v>858</v>
@@ -16902,37 +16948,34 @@
       <c r="L55" t="s">
         <v>775</v>
       </c>
-      <c r="M55" t="s">
-        <v>946</v>
-      </c>
-      <c r="N55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="O55" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>1067</v>
+        <v>1060</v>
       </c>
       <c r="B56" t="s">
-        <v>1068</v>
+        <v>1045</v>
       </c>
       <c r="C56" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D56" t="s">
-        <v>942</v>
-      </c>
-      <c r="E56" t="s">
-        <v>1069</v>
+        <v>894</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>1061</v>
       </c>
       <c r="G56">
         <v>1</v>
       </c>
       <c r="H56" t="s">
-        <v>944</v>
+        <v>896</v>
       </c>
       <c r="I56" t="s">
-        <v>945</v>
+        <v>897</v>
       </c>
       <c r="K56" t="s">
         <v>858</v>
@@ -16941,45 +16984,36 @@
         <v>775</v>
       </c>
       <c r="M56" t="s">
-        <v>991</v>
+        <v>946</v>
       </c>
       <c r="N56">
         <v>0</v>
       </c>
-      <c r="T56" t="s">
-        <v>992</v>
-      </c>
-      <c r="U56" t="s">
-        <v>989</v>
-      </c>
-      <c r="V56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>1070</v>
+        <v>1063</v>
       </c>
       <c r="B57" t="s">
-        <v>1068</v>
+        <v>1045</v>
       </c>
       <c r="C57" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D57" t="s">
-        <v>862</v>
-      </c>
-      <c r="E57" t="s">
-        <v>989</v>
+        <v>1064</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>1065</v>
       </c>
       <c r="G57">
         <v>1</v>
       </c>
       <c r="H57" t="s">
-        <v>864</v>
+        <v>1066</v>
       </c>
       <c r="I57" t="s">
-        <v>865</v>
+        <v>990</v>
       </c>
       <c r="K57" t="s">
         <v>858</v>
@@ -16988,16 +17022,16 @@
         <v>775</v>
       </c>
       <c r="M57" t="s">
-        <v>885</v>
+        <v>991</v>
       </c>
       <c r="N57">
         <v>0</v>
       </c>
       <c r="T57" t="s">
-        <v>886</v>
+        <v>992</v>
       </c>
       <c r="U57" t="s">
-        <v>958</v>
+        <v>989</v>
       </c>
       <c r="V57">
         <v>1</v>
@@ -17005,7 +17039,7 @@
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
       <c r="B58" t="s">
         <v>1068</v>
@@ -17014,19 +17048,19 @@
         <v>24</v>
       </c>
       <c r="D58" t="s">
-        <v>882</v>
+        <v>942</v>
       </c>
       <c r="E58" t="s">
-        <v>958</v>
+        <v>1069</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H58" t="s">
-        <v>884</v>
+        <v>944</v>
       </c>
       <c r="I58" t="s">
-        <v>878</v>
+        <v>945</v>
       </c>
       <c r="K58" t="s">
         <v>858</v>
@@ -17035,19 +17069,16 @@
         <v>775</v>
       </c>
       <c r="M58" t="s">
-        <v>866</v>
+        <v>885</v>
       </c>
       <c r="N58">
         <v>0</v>
       </c>
-      <c r="O58">
-        <v>1</v>
-      </c>
       <c r="T58" t="s">
-        <v>1077</v>
+        <v>886</v>
       </c>
       <c r="U58" t="s">
-        <v>1074</v>
+        <v>958</v>
       </c>
       <c r="V58">
         <v>1</v>
@@ -17055,7 +17086,7 @@
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="B59" t="s">
         <v>1068</v>
@@ -17064,19 +17095,19 @@
         <v>24</v>
       </c>
       <c r="D59" t="s">
-        <v>1073</v>
+        <v>862</v>
       </c>
       <c r="E59" t="s">
-        <v>1074</v>
+        <v>989</v>
       </c>
       <c r="G59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H59" t="s">
-        <v>1075</v>
+        <v>864</v>
       </c>
       <c r="I59" t="s">
-        <v>1076</v>
+        <v>865</v>
       </c>
       <c r="K59" t="s">
         <v>858</v>
@@ -17085,18 +17116,27 @@
         <v>775</v>
       </c>
       <c r="M59" t="s">
-        <v>905</v>
+        <v>866</v>
       </c>
       <c r="N59">
         <v>0</v>
       </c>
-      <c r="P59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="O59">
+        <v>1</v>
+      </c>
+      <c r="T59" t="s">
+        <v>1077</v>
+      </c>
+      <c r="U59" t="s">
+        <v>1074</v>
+      </c>
+      <c r="V59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>1078</v>
+        <v>1071</v>
       </c>
       <c r="B60" t="s">
         <v>1068</v>
@@ -17105,19 +17145,19 @@
         <v>24</v>
       </c>
       <c r="D60" t="s">
-        <v>949</v>
+        <v>882</v>
       </c>
       <c r="E60" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H60" t="s">
-        <v>951</v>
+        <v>884</v>
       </c>
       <c r="I60" t="s">
-        <v>990</v>
+        <v>878</v>
       </c>
       <c r="K60" t="s">
         <v>858</v>
@@ -17126,24 +17166,18 @@
         <v>775</v>
       </c>
       <c r="M60" t="s">
-        <v>1001</v>
+        <v>905</v>
       </c>
       <c r="N60">
         <v>0</v>
       </c>
-      <c r="T60" s="3" t="s">
-        <v>1059</v>
-      </c>
-      <c r="U60" s="3" t="s">
-        <v>1057</v>
-      </c>
-      <c r="V60" s="3">
-        <v>1</v>
+      <c r="P60">
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>1122</v>
+        <v>1072</v>
       </c>
       <c r="B61" t="s">
         <v>1068</v>
@@ -17152,121 +17186,121 @@
         <v>24</v>
       </c>
       <c r="D61" t="s">
-        <v>1123</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>1128</v>
+        <v>1073</v>
+      </c>
+      <c r="E61" t="s">
+        <v>1074</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H61" t="s">
-        <v>1124</v>
+        <v>1075</v>
       </c>
       <c r="I61" t="s">
-        <v>1127</v>
-      </c>
-      <c r="J61" t="s">
-        <v>1125</v>
+        <v>1076</v>
       </c>
       <c r="K61" t="s">
-        <v>1126</v>
-      </c>
-      <c r="T61" s="3"/>
-      <c r="U61" s="3"/>
-      <c r="V61" s="3"/>
-    </row>
-    <row r="62" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+        <v>858</v>
+      </c>
+      <c r="L61" t="s">
+        <v>775</v>
+      </c>
+      <c r="M61" t="s">
+        <v>1001</v>
+      </c>
+      <c r="N61">
+        <v>0</v>
+      </c>
+      <c r="T61" s="3" t="s">
+        <v>1059</v>
+      </c>
+      <c r="U61" s="3" t="s">
+        <v>1057</v>
+      </c>
+      <c r="V61" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" ht="380" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B62" t="s">
         <v>1068</v>
       </c>
       <c r="C62" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D62" t="s">
-        <v>974</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>1057</v>
+        <v>949</v>
+      </c>
+      <c r="E62" t="s">
+        <v>954</v>
       </c>
       <c r="G62">
         <v>1</v>
       </c>
       <c r="H62" t="s">
-        <v>976</v>
+        <v>951</v>
       </c>
       <c r="I62" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="K62" t="s">
         <v>858</v>
       </c>
-      <c r="L62" t="s">
-        <v>775</v>
-      </c>
-      <c r="M62" t="s">
-        <v>1058</v>
-      </c>
-      <c r="N62">
-        <v>0</v>
-      </c>
-      <c r="O62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="T62" s="3"/>
+      <c r="U62" s="3"/>
+      <c r="V62" s="3"/>
+    </row>
+    <row r="63" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>1080</v>
+        <v>1122</v>
       </c>
       <c r="B63" t="s">
         <v>1068</v>
       </c>
       <c r="C63" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D63" t="s">
-        <v>998</v>
-      </c>
-      <c r="E63" t="s">
-        <v>999</v>
+        <v>1123</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>1128</v>
       </c>
       <c r="G63">
         <v>1</v>
       </c>
       <c r="H63" t="s">
-        <v>890</v>
+        <v>1124</v>
       </c>
       <c r="I63" t="s">
-        <v>1000</v>
+        <v>1127</v>
+      </c>
+      <c r="J63" t="s">
+        <v>1125</v>
       </c>
       <c r="K63" t="s">
-        <v>858</v>
+        <v>1126</v>
       </c>
       <c r="L63" t="s">
         <v>775</v>
       </c>
       <c r="M63" t="s">
-        <v>1020</v>
+        <v>1058</v>
       </c>
       <c r="N63">
         <v>0</v>
       </c>
-      <c r="T63" t="s">
-        <v>1084</v>
-      </c>
-      <c r="U63" t="s">
-        <v>1061</v>
-      </c>
-      <c r="V63">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="O63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="B64" t="s">
         <v>1068</v>
@@ -17275,19 +17309,19 @@
         <v>30</v>
       </c>
       <c r="D64" t="s">
-        <v>894</v>
-      </c>
-      <c r="E64" t="s">
-        <v>1082</v>
+        <v>974</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>1057</v>
       </c>
       <c r="G64">
         <v>1</v>
       </c>
       <c r="H64" t="s">
-        <v>896</v>
+        <v>976</v>
       </c>
       <c r="I64" t="s">
-        <v>1083</v>
+        <v>995</v>
       </c>
       <c r="K64" t="s">
         <v>858</v>
@@ -17295,19 +17329,25 @@
       <c r="L64" t="s">
         <v>775</v>
       </c>
+      <c r="M64" t="s">
+        <v>1020</v>
+      </c>
+      <c r="N64">
+        <v>0</v>
+      </c>
       <c r="T64" t="s">
-        <v>1021</v>
+        <v>1084</v>
       </c>
       <c r="U64" t="s">
-        <v>1018</v>
+        <v>1061</v>
       </c>
       <c r="V64">
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>1085</v>
+        <v>1080</v>
       </c>
       <c r="B65" t="s">
         <v>1068</v>
@@ -17316,27 +17356,39 @@
         <v>30</v>
       </c>
       <c r="D65" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>1018</v>
+        <v>998</v>
+      </c>
+      <c r="E65" t="s">
+        <v>999</v>
       </c>
       <c r="G65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H65" t="s">
-        <v>1019</v>
+        <v>890</v>
       </c>
       <c r="I65" t="s">
-        <v>878</v>
+        <v>1000</v>
       </c>
       <c r="K65" t="s">
         <v>858</v>
       </c>
-    </row>
-    <row r="66" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="L65" t="s">
+        <v>775</v>
+      </c>
+      <c r="T65" t="s">
+        <v>1021</v>
+      </c>
+      <c r="U65" t="s">
+        <v>1018</v>
+      </c>
+      <c r="V65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>1115</v>
+        <v>1081</v>
       </c>
       <c r="B66" t="s">
         <v>1068</v>
@@ -17345,25 +17397,83 @@
         <v>30</v>
       </c>
       <c r="D66" t="s">
+        <v>894</v>
+      </c>
+      <c r="E66" t="s">
+        <v>1082</v>
+      </c>
+      <c r="G66">
+        <v>1</v>
+      </c>
+      <c r="H66" t="s">
+        <v>896</v>
+      </c>
+      <c r="I66" t="s">
+        <v>1083</v>
+      </c>
+      <c r="K66" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B67" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C67" t="s">
+        <v>30</v>
+      </c>
+      <c r="D67" t="s">
+        <v>1017</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>1018</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67" t="s">
+        <v>1019</v>
+      </c>
+      <c r="I67" t="s">
+        <v>878</v>
+      </c>
+      <c r="K67" t="s">
+        <v>858</v>
+      </c>
+      <c r="L67" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="68" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B68" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C68" t="s">
+        <v>30</v>
+      </c>
+      <c r="D68" t="s">
         <v>1116</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="E68" s="3" t="s">
         <v>1121</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F68" t="s">
         <v>1117</v>
       </c>
-      <c r="G66">
-        <v>1</v>
-      </c>
-      <c r="I66" t="s">
+      <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="I68" t="s">
         <v>1120</v>
       </c>
-      <c r="K66" t="s">
+      <c r="K68" t="s">
         <v>1118</v>
-      </c>
-      <c r="L66" t="s">
-        <v>1119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>